<commit_message>
HOLDER-EXPORT: partly-in-print column keeps the OR references the audits name; outputs regenerated
print_clauses: 'printed' accepted except before book nouns (printed correspondence/papers/...), the
clause split no longer cuts inside parentheses (split_top), the reviewer-label filter is case-sensitive
and hyphen-bound ('propellers' no longer reads as the label PROP-). E62, E66, E104, E106, E122, E143,
E162, N2-BN, N2-CE, N2-CJ now carry their printed reply/request/context reference. New regression test
(10 OK). Delivery regenerated from origin/main 124430116 (69 rows; drift unchanged: E96 now N2).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0198Cv8ypBfBVfRToKVWx33M
</commit_message>
<xml_diff>
--- a/outreach/huntington-delivery/huntington-decipherments-2026-10.xlsx
+++ b/outreach/huntington-delivery/huntington-decipherments-2026-10.xlsx
@@ -2680,7 +2680,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>OR I/33 p.814 prints Biggs's same-day reply on the coal and Salvor, not this telegram.</t>
+          <t>OR I/33 p.814 prints Biggs's same-day reply on the coal and Salvor, not this telegram. Purple = 1,000 (tons) and Appian/Animal = Monroe agree with Biggs's printed same-day offer (OR I/33 p.814).</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -3345,7 +3345,11 @@
           <t>Not found in the Official Records (ser. I and III by date and correspondent), the Huntington collection's full text, Internet Archive full text, Google Books, OpenAlex or CORE (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Biggs's printed replies of 5 Apr (OR I/35 pt 2 pp.37-38, the Montauk and two other propellers) and 6 Apr (OR I/33 p.814, Montauk's broken valve-crank, Spaulding not yet arrived) answer the ships and orders this telegram names.</t>
+        </is>
+      </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -3907,7 +3911,11 @@
           <t>Not found in the Official Records (Army and Navy, by date and correspondent), Internet Archive full text, Google Books, OpenAlex, Semantic Scholar or CORE (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Van Vliet's printed replies of 3 Jan 1865 to Meigs (OR I/46 pt 2 p.28, steamers available at New York) answer this telegram and fix its year.</t>
+        </is>
+      </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -4095,7 +4103,7 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>the order it answers is printed (Humphreys to Benham 29 Feb 1864, OR I/33 pp.616-617).</t>
+          <t>Humphreys' printed order of 29 Feb 1864 (OR I/33 pp.616-617: advance guard train, canvas pontoons, 42 chesses per chess-wagon) matches the date [29], [Advance] and [42].</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
@@ -4938,7 +4946,11 @@
           <t>Not found in the Official Records (ser. I vols. 42 pt 2, 43 pts 1-2), the Grant Papers (vol. 11), Internet Archive full text, Google Books or the Huntington's own full-text search (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>printed sibling Meigs to Ingalls 6 Aug 1864 (OR I/42 pt 2 p.66).</t>
+        </is>
+      </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5120,7 +5132,11 @@
           <t>Not found in the Official Records (ser. I vols. 42 pt 3, 44), the Grant Papers (vol. 13, snippet search), Internet Archive full text or Google Books (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>Grant's printed telegram to Meigs of 19 Dec 1864 (OR ser. I vol. 44 p.755) records that he had 'directed General Ingalls to go on'.</t>
+        </is>
+      </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5310,7 +5326,11 @@
           <t>Not found in OR ser. I vols. 40 pt 2, 34, ser. III vol. 4, Internet Archive full text or Google Books (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>context printed (Halleck to Canby 24 June 1864, OR I/34 pt 4; Ingalls 26-27 June, OR I/40 pt 2), not E143's instructions.</t>
+        </is>
+      </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5593,7 +5613,11 @@
           <t>Not found in the Official Records (ser. I vol. 37 pt 1), Internet Archive full text, Google Books or the Huntington's full-text search (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Hunter's printed request of 21-22 May for two brigadiers (OR I/37 pt 1 pp.516-517) and the reply actually sent, E9 (OR I/37 pt 1 p.525).</t>
+        </is>
+      </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5686,7 +5710,11 @@
           <t>Not found in the Official Records (ser. I vol. 43), Internet Archive full text, Google Books or the Huntington's full-text search (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Sheridan's printed request for 100 Spencer rifles, approved 21 Aug (OR I/43 pt 1 p.860).</t>
+        </is>
+      </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5779,7 +5807,11 @@
           <t>Not found in the Official Records (ser. I vol. 33), Internet Archive full text or Google Books (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Humphreys's printed 10 AM telegram on the scouts' return (OR I/33 p.639), which E104 answers.</t>
+        </is>
+      </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>
@@ -5872,7 +5904,11 @@
           <t>Not found in the Official Records (ser. I vols. 42-43), Butler's Book (1892), Butler's printed correspondence (vols. III-V), Chronicling America, Internet Archive full text, Google Books or the Huntington's full-text search (searched 8 Oct 2026).</t>
         </is>
       </c>
-      <c r="P58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Butler's printed call of 2 Nov for two batteries of Napoleons and Hawley's report that Battery M, 1st U.S. (six light 12s) went to New York (OR I/42 pt 3 p.489; I/43 pt 2 p.559).</t>
+        </is>
+      </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
           <t>N3: no prior plaintext or decipherment located after a logged search; checked by two independent audits</t>

</xml_diff>